<commit_message>
feat: implement stock monitoring logic and initialize historical data and output files
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260211.xlsx
+++ b/outputs/monitor_xlsx/20260211.xlsx
@@ -999,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2388,13 +2388,13 @@
         <v>717</v>
       </c>
       <c r="L24" t="n">
-        <v>4437</v>
+        <v>3539</v>
       </c>
       <c r="M24" t="n">
         <v>-106283</v>
       </c>
       <c r="N24" t="n">
-        <v>3.75</v>
+        <v>3.73</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2452,6 +2452,59 @@
       <c r="O25" t="inlineStr">
         <is>
           <t>偏多</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>6515</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>穎崴</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5005</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E26" t="n">
+        <v>384</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>-18</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-97</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>48</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>339</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1648</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-8884</v>
+      </c>
+      <c r="N26" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>偏空</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement intraday monitor and update global market data tracking
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260211.xlsx
+++ b/outputs/monitor_xlsx/20260211.xlsx
@@ -481,7 +481,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -824,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -880,7 +878,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1002,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2426,6 +2423,51 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3167</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>大量</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>271.5</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10013</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="G27" t="n">
+        <v>7980</v>
+      </c>
+      <c r="H27" t="n">
+        <v>95</v>
+      </c>
+      <c r="I27" t="n">
+        <v>475</v>
+      </c>
+      <c r="J27" t="n">
+        <v>272</v>
+      </c>
+      <c r="K27" t="n">
+        <v>6004</v>
+      </c>
+      <c r="L27" t="n">
+        <v>11851</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-21379</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>

</xml_diff>